<commit_message>
weibull - fixed large file issue
</commit_message>
<xml_diff>
--- a/Experiments_Summary.xlsx
+++ b/Experiments_Summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
   <si>
     <t>Model_Name</t>
   </si>
@@ -46,10 +46,43 @@
     <t>Test_Balanced_Accuracy</t>
   </si>
   <si>
+    <t>Learning_Rate_Head</t>
+  </si>
+  <si>
+    <t>Total_Folds</t>
+  </si>
+  <si>
+    <t>Avg_Test_AUROC</t>
+  </si>
+  <si>
+    <t>Avg_Test_F1_Score</t>
+  </si>
+  <si>
+    <t>Avg_Test_Balanced_Accuracy</t>
+  </si>
+  <si>
+    <t>Avg_Test_CIndex</t>
+  </si>
+  <si>
     <t>whole_slice</t>
   </si>
   <si>
     <t>/nas-ctm01/datasets/public/medical_datasets/lung_ct_datasets/nlst/preprocessed_data/protocol_5/2d/ws</t>
+  </si>
+  <si>
+    <t>lung</t>
+  </si>
+  <si>
+    <t>/nas-ctm01/datasets/public/medical_datasets/lung_ct_datasets/nlst/preprocessed_data/protocol_5/2d/lung</t>
+  </si>
+  <si>
+    <t>/nas-ctm01/datasets/public/medical_datasets/lung_ct_datasets/nlst/preprocessed_data/protocol_5/2d/masked</t>
+  </si>
+  <si>
+    <t>masked</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
 </sst>
 </file>
@@ -120,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -140,11 +173,29 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -451,22 +502,28 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="8" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="15" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -497,13 +554,31 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="C2" s="5">
         <v>0.0001</v>
@@ -528,6 +603,562 @@
       </c>
       <c r="J2" s="5">
         <v>0.629539966583252</v>
+      </c>
+      <c r="K2" s="7"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+      <c r="A3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D3" s="6">
+        <v>200</v>
+      </c>
+      <c r="E3" s="6">
+        <v>32</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G3" s="6">
+        <v>22</v>
+      </c>
+      <c r="H3" s="5">
+        <v>0.6900726556777954</v>
+      </c>
+      <c r="I3" s="5">
+        <v>0.5128205418586731</v>
+      </c>
+      <c r="J3" s="5">
+        <v>0.6702986359596252</v>
+      </c>
+      <c r="K3" s="7"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D4" s="6">
+        <v>200</v>
+      </c>
+      <c r="E4" s="6">
+        <v>32</v>
+      </c>
+      <c r="F4" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G4" s="6">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5">
+        <v>0.698143720626831</v>
+      </c>
+      <c r="I4" s="5">
+        <v>0.4347825944423676</v>
+      </c>
+      <c r="J4" s="5">
+        <v>0.6109765768051147</v>
+      </c>
+      <c r="K4" s="7"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+      <c r="A5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="D5" s="6">
+        <v>100</v>
+      </c>
+      <c r="E5" s="6">
+        <v>32</v>
+      </c>
+      <c r="F5" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G5" s="6">
+        <v>22</v>
+      </c>
+      <c r="H5" s="5">
+        <v>0.646489143371582</v>
+      </c>
+      <c r="I5" s="5">
+        <v>0.3888888955116272</v>
+      </c>
+      <c r="J5" s="5">
+        <v>0.598870038986206</v>
+      </c>
+      <c r="K5" s="7"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+      <c r="A6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D6" s="6">
+        <v>200</v>
+      </c>
+      <c r="E6" s="6">
+        <v>32</v>
+      </c>
+      <c r="F6" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G6" s="6">
+        <v>22</v>
+      </c>
+      <c r="H6" s="5">
+        <v>0.6311541795730591</v>
+      </c>
+      <c r="I6" s="5">
+        <v>0.3902438879013062</v>
+      </c>
+      <c r="J6" s="5">
+        <v>0.5887812972068787</v>
+      </c>
+      <c r="K6" s="7"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D7" s="6">
+        <v>200</v>
+      </c>
+      <c r="E7" s="6">
+        <v>32</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G7" s="6">
+        <v>22</v>
+      </c>
+      <c r="H7" s="5">
+        <v>0.6311541795730591</v>
+      </c>
+      <c r="I7" s="5">
+        <v>0.3902438879013062</v>
+      </c>
+      <c r="J7" s="5">
+        <v>0.5887812972068787</v>
+      </c>
+      <c r="K7" s="7"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="9"/>
+      <c r="D8" s="6">
+        <v>2</v>
+      </c>
+      <c r="E8" s="6">
+        <v>32</v>
+      </c>
+      <c r="F8" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G8" s="6">
+        <v>22</v>
+      </c>
+      <c r="H8" s="5">
+        <v>0.5423728823661804</v>
+      </c>
+      <c r="I8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="K8" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="L8" s="8"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="9"/>
+      <c r="D9" s="6">
+        <v>200</v>
+      </c>
+      <c r="E9" s="6">
+        <v>32</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G9" s="6">
+        <v>22</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0.6989508271217346</v>
+      </c>
+      <c r="I9" s="5">
+        <v>0.4255319237709045</v>
+      </c>
+      <c r="J9" s="5">
+        <v>0.6025020480155945</v>
+      </c>
+      <c r="K9" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="L9" s="8"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
+      <c r="A10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D10" s="6">
+        <v>200</v>
+      </c>
+      <c r="E10" s="6">
+        <v>32</v>
+      </c>
+      <c r="F10" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G10" s="6">
+        <v>22</v>
+      </c>
+      <c r="H10" s="5">
+        <v>0.6311541795730591</v>
+      </c>
+      <c r="I10" s="5">
+        <v>0.3902438879013062</v>
+      </c>
+      <c r="J10" s="5">
+        <v>0.5887812972068787</v>
+      </c>
+      <c r="K10" s="7"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="D11" s="6">
+        <v>2</v>
+      </c>
+      <c r="E11" s="6">
+        <v>32</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G11" s="6">
+        <v>22</v>
+      </c>
+      <c r="H11" s="5">
+        <v>0.5900000333786011</v>
+      </c>
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="K11" s="7"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D12" s="6">
+        <v>100</v>
+      </c>
+      <c r="E12" s="6">
+        <v>32</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G12" s="6">
+        <v>22</v>
+      </c>
+      <c r="H12" s="5">
+        <v>0.7233333587646484</v>
+      </c>
+      <c r="I12" s="5">
+        <v>0.5106382966041565</v>
+      </c>
+      <c r="J12" s="5">
+        <v>0.675000011920929</v>
+      </c>
+      <c r="K12" s="7"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
+      <c r="A13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="D13" s="6">
+        <v>100</v>
+      </c>
+      <c r="E13" s="6">
+        <v>32</v>
+      </c>
+      <c r="F13" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="G13" s="6">
+        <v>22</v>
+      </c>
+      <c r="H13" s="5">
+        <v>0.7274999618530273</v>
+      </c>
+      <c r="I13" s="5">
+        <v>0.5</v>
+      </c>
+      <c r="J13" s="5">
+        <v>0.6666666269302368</v>
+      </c>
+      <c r="K13" s="7"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
+      <c r="A14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="6">
+        <v>22</v>
+      </c>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="6">
+        <v>3</v>
+      </c>
+      <c r="M14" s="5">
+        <v>0.674999992052714</v>
+      </c>
+      <c r="N14" s="5">
+        <v>0.4004127979278564</v>
+      </c>
+      <c r="O14" s="5">
+        <v>0.6055555542310079</v>
+      </c>
+      <c r="P14" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
+      <c r="A15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="6">
+        <v>22</v>
+      </c>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="6">
+        <v>3</v>
+      </c>
+      <c r="M15" s="5">
+        <v>0.6874999602635702</v>
+      </c>
+      <c r="N15" s="5">
+        <v>0.4707868993282318</v>
+      </c>
+      <c r="O15" s="5">
+        <v>0.6444444259007772</v>
+      </c>
+      <c r="P15" s="8"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
+      <c r="A16" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="5">
+        <v>0.00001</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="6">
+        <v>22</v>
+      </c>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="6">
+        <v>3</v>
+      </c>
+      <c r="M16" s="5">
+        <v>0.5086419582366943</v>
+      </c>
+      <c r="N16" s="6">
+        <v>0</v>
+      </c>
+      <c r="O16" s="6">
+        <v>0</v>
+      </c>
+      <c r="P16" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
+      <c r="A17" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="5">
+        <v>0.0001</v>
+      </c>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="6">
+        <v>22</v>
+      </c>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="6">
+        <v>3</v>
+      </c>
+      <c r="M17" s="5">
+        <v>0.6929012537002563</v>
+      </c>
+      <c r="N17" s="6">
+        <v>0</v>
+      </c>
+      <c r="O17" s="6">
+        <v>0</v>
+      </c>
+      <c r="P17" s="6">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more efficient code plus radioFM
</commit_message>
<xml_diff>
--- a/Experiments_Summary.xlsx
+++ b/Experiments_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1277,7 +1277,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Binary_ws</t>
+          <t>Binary_lung</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1290,38 +1290,1486 @@
         <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>0.6724999944368998</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>0.7180555462837219</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.3065453668435414</v>
+      </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
-        <v>0.6361111203829447</v>
+        <v>0.5944444537162781</v>
       </c>
       <c r="I15" t="n">
-        <v>0.461451252301534</v>
+        <v>0.3705882330735524</v>
       </c>
       <c r="J15" t="n">
-        <v>0.04972610417041414</v>
-      </c>
-      <c r="K15" t="inlineStr"/>
+        <v>0.0177473625427014</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.008404500681152147</v>
+      </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="n">
-        <v>0.03215509072213786</v>
+        <v>0.04374447422688386</v>
       </c>
       <c r="N15" t="n">
-        <v>0.03891383121269985</v>
+        <v>0.08668573726387595</v>
       </c>
       <c r="O15" t="n">
+        <v>0.5944444537162781</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.04374447422688386</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0.611289362112681</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0.04465261233339038</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Binary_ws</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C16" t="n">
+        <v>22</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.6802777449289957</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.3292898635069529</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0.6111111044883728</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.4248851239681244</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.0462597515408647</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0.0445713789914697</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="n">
+        <v>0.04530416812354012</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0.0580141072311248</v>
+      </c>
+      <c r="O16" t="n">
+        <v>0.6111111044883728</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.04530416812354012</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.6057166258494059</v>
+      </c>
+      <c r="R16" t="n">
+        <v>0.046444056459004</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Binary_ws_unfrozen</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C17" t="n">
+        <v>22</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.6694444219271342</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.3532979488372803</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>0.6194444298744202</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.4214214285214742</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.0302790475087229</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0.020371539477665</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="n">
+        <v>0.03868995764163432</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.06460916600228836</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0.6194444298744202</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0.03868995764163432</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.6372597614924113</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0.0426971189543995</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Binary_lung_unfrozen</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C18" t="n">
+        <v>22</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.761388878027598</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.285064438978831</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0.6777777671813965</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.5158483982086182</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.01979444973510131</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.01932911187972722</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="n">
+        <v>0.0171234074691646</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.02356130428270595</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.6777777671813965</v>
+      </c>
+      <c r="P18" t="n">
+        <v>0.0171234074691646</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.6824351747830709</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.02547267761211013</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Binary_masked</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C19" t="n">
+        <v>22</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.7374999721844991</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.2901187737782796</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0.6388888955116272</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.4489954610665639</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.008686954775978832</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.00939480916770619</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="n">
+        <v>0.07647722305038354</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.1283333211564751</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.6388888955116272</v>
+      </c>
+      <c r="P19" t="n">
+        <v>0.07647722305038354</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.6467669606208801</v>
+      </c>
+      <c r="R19" t="n">
+        <v>0.07412415624564839</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Binary_masked_unfrozen</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C20" t="n">
+        <v>22</v>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.7530555327733358</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.2977002759774526</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>0.6250000397364298</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.4206773738066356</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.05390462990124372</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.04140699839998828</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="n">
+        <v>0.05314202337176079</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.08833876738283358</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.6250000397364298</v>
+      </c>
+      <c r="P20" t="n">
+        <v>0.05314202337176079</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>0.6376960674921671</v>
+      </c>
+      <c r="R20" t="n">
+        <v>0.02982949637940507</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Binary_ws</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C21" t="n">
+        <v>22</v>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.6750000317891439</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.5352539817492167</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0.6444444457689921</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.472810963789622</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.04876738852446711</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.04299898082445552</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="n">
+        <v>0.04101338115208705</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.05243174356704906</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.6444444457689921</v>
+      </c>
+      <c r="P21" t="n">
+        <v>0.04101338115208705</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0.6404328147570292</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.04775576276599745</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Binary_ws</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C22" t="n">
+        <v>22</v>
+      </c>
+      <c r="D22" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.6777777473131815</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.5347485542297363</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.50533127784729</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.04998857642828167</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.04312062077190951</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="n">
+        <v>0.06905444741871394</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.09493238731669183</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P22" t="n">
+        <v>0.06905444741871394</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0.6619555552800497</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.07178272167197755</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C23" t="n">
+        <v>22</v>
+      </c>
+      <c r="D23" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.6750000317891439</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.5352539817492167</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0.569444457689921</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.2883597960074742</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.04876738852446711</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.04299898082445552</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="n">
+        <v>0.02389535058159446</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.05511287742699388</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.569444457689921</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.02389535058159446</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>0.6483565370241801</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.04559983856047613</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C24" t="n">
+        <v>22</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.6750000317891439</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.5352539817492167</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
         <v>0.6361111203829447</v>
       </c>
-      <c r="P15" t="n">
-        <v>0.03215509072213786</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0.6214166482289633</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0.03341367063597313</v>
+      <c r="I24" t="n">
+        <v>0.4512180785338084</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.04876738852446711</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.04299898082445552</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="n">
+        <v>0.03491611882203919</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.05617007846464612</v>
+      </c>
+      <c r="O24" t="n">
+        <v>0.6361111203829447</v>
+      </c>
+      <c r="P24" t="n">
+        <v>0.03491611882203919</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0.6701036890347799</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.05639690825394791</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C25" t="n">
+        <v>22</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.6040123303731283</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.4023249844710032</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.3925263384977977</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.01680890165551272</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.0877760461480723</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="n">
+        <v>0.01571348308978993</v>
+      </c>
+      <c r="N25" t="n">
+        <v>0.02491096407036001</v>
+      </c>
+      <c r="O25" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="P25" t="n">
+        <v>0.01571348308978993</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0.5779856642087301</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0.01715543494942115</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C26" t="n">
+        <v>22</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.6308641831080118</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.4101592103640239</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>0.5555555621782938</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.3464452524979909</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.01176893225703141</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.08217685279196114</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="n">
+        <v>0.03747428387082062</v>
+      </c>
+      <c r="N26" t="n">
+        <v>0.04184199902328577</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.5555555621782938</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.03747428387082062</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0.554495096206665</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.03799833592158253</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C27" t="n">
+        <v>22</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.7669753233591715</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.6636340618133545</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0.6583333214124044</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.4850857555866241</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.02187661595596984</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.03857056303696577</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="n">
+        <v>0.01360828770443337</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.0222654709887029</v>
+      </c>
+      <c r="O27" t="n">
+        <v>0.6583333214124044</v>
+      </c>
+      <c r="P27" t="n">
+        <v>0.01360828770443337</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0.6706487735112509</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0.007504073290785176</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C28" t="n">
+        <v>22</v>
+      </c>
+      <c r="D28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.554938276608785</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.547889788945516</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0.5388888915379842</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.187600647409757</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.03448238791338994</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.005337050282270258</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="n">
+        <v>0.003928395358104403</v>
+      </c>
+      <c r="N28" t="n">
+        <v>0.02465924648509743</v>
+      </c>
+      <c r="O28" t="n">
+        <v>0.5388888915379842</v>
+      </c>
+      <c r="P28" t="n">
+        <v>0.003928395358104403</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0.6486254930496216</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0.04989722428412248</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C29" t="n">
+        <v>22</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.4574073950449626</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.4763709902763367</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>0.497222234805425</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.1413817678888639</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.03725243515284618</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.02611922751504557</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="n">
+        <v>0.03215510874383116</v>
+      </c>
+      <c r="N29" t="n">
+        <v>0.06043857519630202</v>
+      </c>
+      <c r="O29" t="n">
+        <v>0.497222234805425</v>
+      </c>
+      <c r="P29" t="n">
+        <v>0.03215510874383116</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0.5012608965237936</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.06831620322264773</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C30" t="n">
+        <v>22</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.4675925970077515</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.4548900624116262</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0.4888888796170552</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.08024691541989644</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.06053318116116507</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.06051284787483691</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="n">
+        <v>0.0321550855730742</v>
+      </c>
+      <c r="N30" t="n">
+        <v>0.06818124292876049</v>
+      </c>
+      <c r="O30" t="n">
+        <v>0.4888888796170552</v>
+      </c>
+      <c r="P30" t="n">
+        <v>0.0321550855730742</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0.4798457225163777</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0.1115330794236924</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ws</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C31" t="n">
+        <v>22</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.4666666487852733</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.4533737599849701</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>0.4805555641651154</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.09611993034680684</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.03998312804202871</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.04290529784879946</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="n">
+        <v>0.04101340806499109</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0.08885984050050091</v>
+      </c>
+      <c r="O31" t="n">
+        <v>0.4805555641651154</v>
+      </c>
+      <c r="P31" t="n">
+        <v>0.04101340806499109</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0.4572823643684387</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0.0858000446282922</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>lung_radio_frozen</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C32" t="n">
+        <v>22</v>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.6061728398005167</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.5936315457026163</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.1242708389957746</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.4216248492399852</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.0520187809289429</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.02796602883009606</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.002620993199262494</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="N32" t="n">
+        <v>0.02483285144258953</v>
+      </c>
+      <c r="O32" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="P32" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0.5647678772608439</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0.01940908164067787</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>lung_radio_unfrozen</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C33" t="n">
+        <v>22</v>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.5993827184041342</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.5718979040781657</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.1262166673938433</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.3978034754594167</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.02264682721450439</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.01030885992897227</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.001969844602953353</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0.03545061676519656</v>
+      </c>
+      <c r="O33" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="P33" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0.5580615599950155</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.01112326027637736</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>masked_radio_frozen</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C34" t="n">
+        <v>22</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.6061728398005167</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.5936315457026163</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.1242708389957746</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.4216248492399852</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.0520187809289429</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.02796602883009606</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.002620993199262494</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="N34" t="n">
+        <v>0.02483285144258953</v>
+      </c>
+      <c r="O34" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="P34" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0.5647678772608439</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.01940908164067787</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ws_radio_frozen</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C35" t="n">
+        <v>22</v>
+      </c>
+      <c r="D35" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.6061728398005167</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.5936315457026163</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.1242708389957746</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0.4216248492399852</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.0520187809289429</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.02796602883009606</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0.002620993199262494</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="N35" t="n">
+        <v>0.02483285144258953</v>
+      </c>
+      <c r="O35" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="P35" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0.5647678772608439</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0.01940908164067787</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>masked_radio_unfrozen</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C36" t="n">
+        <v>22</v>
+      </c>
+      <c r="D36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.5993827184041342</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.5718979040781657</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.1262166673938433</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.3978034754594167</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.02264682721450439</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.01030885992897227</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.001969844602953353</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0.03545061676519656</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0.5580615599950155</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0.01112326027637736</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ws_radio_unfrozen</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C37" t="n">
+        <v>22</v>
+      </c>
+      <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.5993827184041342</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.5718979040781657</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.1262166673938433</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.3978034754594167</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.02264682721450439</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.01030885992897227</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.001969844602953353</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="N37" t="n">
+        <v>0.03545061676519656</v>
+      </c>
+      <c r="O37" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="P37" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0.5580615599950155</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0.01112326027637736</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>lung_unfrozen_med_reg_64</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C38" t="n">
+        <v>22</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.7583333253860474</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.6909274657567342</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.1151315396030744</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.6861111124356588</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.5204678376515707</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.03704476253122629</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.0332223833452473</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.006930309941077968</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.02749861296829705</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0.02894589359930188</v>
+      </c>
+      <c r="O38" t="n">
+        <v>0.6861111124356588</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0.02749861296829705</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>0.6457585493723551</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0.01718248205627023</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>lung_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C39" t="n">
+        <v>22</v>
+      </c>
+      <c r="D39" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.7583333253860474</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.6909274657567342</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.1151315396030744</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.6861111124356588</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.5204678376515707</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.03704476253122629</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.0332223833452473</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.006930309941077968</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.02749861296829705</v>
+      </c>
+      <c r="N39" t="n">
+        <v>0.02894589359930188</v>
+      </c>
+      <c r="O39" t="n">
+        <v>0.6861111124356588</v>
+      </c>
+      <c r="P39" t="n">
+        <v>0.02749861296829705</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0.6457585493723551</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0.01718248205627023</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>lung_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C40" t="n">
+        <v>22</v>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.7515432039896647</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.7065958976745605</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.1104106903076172</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.6222222248713175</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.4110016425450643</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.02656110095530181</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.02696144616643013</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.005783183394275743</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.04631481341638571</v>
+      </c>
+      <c r="N40" t="n">
+        <v>0.09714666605188385</v>
+      </c>
+      <c r="O40" t="n">
+        <v>0.6222222248713175</v>
+      </c>
+      <c r="P40" t="n">
+        <v>0.04631481341638571</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0.6404226024945577</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0.026548026103587</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>lung_unfrozen_med_reg_64</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C41" t="n">
+        <v>22</v>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.7182098627090454</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.6866312821706136</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.1201578105489413</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.6444444457689921</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.4303233077128728</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.01371983956692996</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.009616515688300849</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.003787863766263155</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.06712802507473127</v>
+      </c>
+      <c r="N41" t="n">
+        <v>0.1412710913608317</v>
+      </c>
+      <c r="O41" t="n">
+        <v>0.6444444457689921</v>
+      </c>
+      <c r="P41" t="n">
+        <v>0.06712802507473127</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0.6493601202964783</v>
+      </c>
+      <c r="R41" t="n">
+        <v>0.01006019797878372</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tabular data to text
</commit_message>
<xml_diff>
--- a/Experiments_Summary.xlsx
+++ b/Experiments_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2772,6 +2772,760 @@
         <v>0.01006019797878372</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>masked_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C42" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.779938280582428</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.7212534745534261</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.1108078807592392</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.5454332232475281</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.02417279762807992</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.04139772608022362</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.006992792258105583</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.04138794527037967</v>
+      </c>
+      <c r="N42" t="n">
+        <v>0.04375373816919498</v>
+      </c>
+      <c r="O42" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="P42" t="n">
+        <v>0.04138794527037967</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0.6631452043851217</v>
+      </c>
+      <c r="R42" t="n">
+        <v>0.02760079309767969</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>masked_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C43" t="n">
+        <v>22</v>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.779938280582428</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.7212534745534261</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.1108078807592392</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.5454332232475281</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.02417279762807992</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.04139772608022362</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.006992792258105583</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.04138794527037967</v>
+      </c>
+      <c r="N43" t="n">
+        <v>0.04375373816919498</v>
+      </c>
+      <c r="O43" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="P43" t="n">
+        <v>0.04138794527037967</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>0.6631452043851217</v>
+      </c>
+      <c r="R43" t="n">
+        <v>0.02760079309767969</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>ws_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C44" t="n">
+        <v>22</v>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.750308632850647</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.6972453991572062</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.1102481509248416</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.6472222010294596</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.4727095564206441</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.01026439158585974</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.01590710472105708</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.003657719155071491</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.01712335590034907</v>
+      </c>
+      <c r="N44" t="n">
+        <v>0.02269092807431733</v>
+      </c>
+      <c r="O44" t="n">
+        <v>0.6472222010294596</v>
+      </c>
+      <c r="P44" t="n">
+        <v>0.01712335590034907</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>0.655231237411499</v>
+      </c>
+      <c r="R44" t="n">
+        <v>0.03545959297481422</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ws_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C45" t="n">
+        <v>22</v>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.750308632850647</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.6972453991572062</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.1102481509248416</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.6472222010294596</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.4727095564206441</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.01026439158585974</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.01590710472105708</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.003657719155071491</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.01712335590034907</v>
+      </c>
+      <c r="N45" t="n">
+        <v>0.02269092807431733</v>
+      </c>
+      <c r="O45" t="n">
+        <v>0.6472222010294596</v>
+      </c>
+      <c r="P45" t="n">
+        <v>0.01712335590034907</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>0.655231237411499</v>
+      </c>
+      <c r="R45" t="n">
+        <v>0.03545959297481422</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>lung_radio_frozen</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C46" t="n">
+        <v>22</v>
+      </c>
+      <c r="D46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.5646605292956034</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.5592620571454366</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.1267349819342295</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.5222222208976746</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.3726898034413655</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.06943963216138521</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.03796475431558221</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.0004855356616961235</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.03747426325259959</v>
+      </c>
+      <c r="N46" t="n">
+        <v>0.03862246438014032</v>
+      </c>
+      <c r="O46" t="n">
+        <v>0.5222222208976746</v>
+      </c>
+      <c r="P46" t="n">
+        <v>0.03747426325259959</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>0.5197017788887024</v>
+      </c>
+      <c r="R46" t="n">
+        <v>0.03245576114304535</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>lung_radio_unfrozen</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C47" t="n">
+        <v>22</v>
+      </c>
+      <c r="D47" t="n">
+        <v>3</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.582253078619639</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.5772049427032471</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.1265902022520701</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.5527777671813965</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.2964392999807994</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.01301429476918438</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.02173070685657801</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.01228707093973039</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.01964186439892599</v>
+      </c>
+      <c r="N47" t="n">
+        <v>0.02683911843699489</v>
+      </c>
+      <c r="O47" t="n">
+        <v>0.5527777671813965</v>
+      </c>
+      <c r="P47" t="n">
+        <v>0.01964186439892599</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>0.5816750327746073</v>
+      </c>
+      <c r="R47" t="n">
+        <v>0.04533517937991077</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>masked_radio_frozen</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C48" t="n">
+        <v>22</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.4987654089927673</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.4964619576931</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.135143925746282</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.4750000238418579</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.3736263811588287</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.04364854072333719</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.01793664925001662</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.002920762179963498</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" t="n">
+        <v>0.4750000238418579</v>
+      </c>
+      <c r="P48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>0.4530516564846039</v>
+      </c>
+      <c r="R48" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>masked_radio_unfrozen</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C49" t="n">
+        <v>22</v>
+      </c>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.5231481492519379</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.4823098282019297</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.1288677702347437</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.4833333492279053</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.2490842541058858</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.03062562846201696</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.03731317950051978</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.004134124493627369</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.01178510178061619</v>
+      </c>
+      <c r="N49" t="n">
+        <v>0.176129165165065</v>
+      </c>
+      <c r="O49" t="n">
+        <v>0.4833333492279053</v>
+      </c>
+      <c r="P49" t="n">
+        <v>0.01178510178061619</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0.4270344376564026</v>
+      </c>
+      <c r="R49" t="n">
+        <v>0.03679390372207091</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ws_radio_frozen</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C50" t="n">
+        <v>22</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.6061728398005167</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.5936315457026163</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.1242708389957746</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.4216248492399852</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.0520187809289429</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.02796602883009606</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.002620993199262494</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="N50" t="n">
+        <v>0.02483285144258953</v>
+      </c>
+      <c r="O50" t="n">
+        <v>0.5861111283302307</v>
+      </c>
+      <c r="P50" t="n">
+        <v>0.02576005466145912</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0.5647678772608439</v>
+      </c>
+      <c r="R50" t="n">
+        <v>0.01940908164067787</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>ws_radio_unfrozen</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C51" t="n">
+        <v>22</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.5993827184041342</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.5718979040781657</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.1262166673938433</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.3978034754594167</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.02264682721450439</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.01030885992897227</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.001969844602953353</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="N51" t="n">
+        <v>0.03545061676519656</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0.575000007947286</v>
+      </c>
+      <c r="P51" t="n">
+        <v>0.01800205872188277</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0.5580615599950155</v>
+      </c>
+      <c r="R51" t="n">
+        <v>0.01112326027637736</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>lung_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C52" t="n">
+        <v>22</v>
+      </c>
+      <c r="D52" t="n">
+        <v>3</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.7515432039896647</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.7065958976745605</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.1104106903076172</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.6222222248713175</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.4110016425450643</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.02656110095530181</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.02696144616643013</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.005783183394275743</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.04631481341638571</v>
+      </c>
+      <c r="N52" t="n">
+        <v>0.09714666605188385</v>
+      </c>
+      <c r="O52" t="n">
+        <v>0.6222222248713175</v>
+      </c>
+      <c r="P52" t="n">
+        <v>0.04631481341638571</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0.6404226024945577</v>
+      </c>
+      <c r="R52" t="n">
+        <v>0.026548026103587</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>masked_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C53" t="n">
+        <v>22</v>
+      </c>
+      <c r="D53" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.779938280582428</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.7212534745534261</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.1108078807592392</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.5454332232475281</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.02417279762807992</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.04139772608022362</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.006992792258105583</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.04138794527037967</v>
+      </c>
+      <c r="N53" t="n">
+        <v>0.04375373816919498</v>
+      </c>
+      <c r="O53" t="n">
+        <v>0.7083333333333334</v>
+      </c>
+      <c r="P53" t="n">
+        <v>0.04138794527037967</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0.6631452043851217</v>
+      </c>
+      <c r="R53" t="n">
+        <v>0.02760079309767969</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ws_unfrozen_med_reg_24</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C54" t="n">
+        <v>22</v>
+      </c>
+      <c r="D54" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.750308632850647</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.6972453991572062</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.1102481509248416</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.6472222010294596</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.4727095564206441</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.01026439158585974</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.01590710472105708</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.003657719155071491</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.01712335590034907</v>
+      </c>
+      <c r="N54" t="n">
+        <v>0.02269092807431733</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0.6472222010294596</v>
+      </c>
+      <c r="P54" t="n">
+        <v>0.01712335590034907</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0.655231237411499</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0.03545959297481422</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
late fusion and survival models
</commit_message>
<xml_diff>
--- a/Experiments_Summary.xlsx
+++ b/Experiments_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R117"/>
+  <dimension ref="A1:T129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,16 @@
           <t>Std_Test_precision</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Avg_Test_td_auc</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>std_Test_td_auc</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -577,6 +587,8 @@
       <c r="R2" t="n">
         <v>0.0485919095517561</v>
       </c>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -635,6 +647,8 @@
       <c r="R3" t="n">
         <v>0.05271970781422992</v>
       </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -693,6 +707,8 @@
       <c r="R4" t="n">
         <v>0.04799526486346187</v>
       </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -751,6 +767,8 @@
       <c r="R5" t="n">
         <v>0.02966688568351711</v>
       </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -809,6 +827,8 @@
       <c r="R6" t="n">
         <v>0.05241903603056015</v>
       </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -867,6 +887,8 @@
       <c r="R7" t="n">
         <v>0.01718248205627023</v>
       </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -925,6 +947,8 @@
       <c r="R8" t="n">
         <v>0.05651580495753514</v>
       </c>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -983,6 +1007,8 @@
       <c r="R9" t="n">
         <v>0.04353825330072314</v>
       </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1041,6 +1067,8 @@
       <c r="R10" t="n">
         <v>0.01669251672497994</v>
       </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1099,6 +1127,8 @@
       <c r="R11" t="n">
         <v>0.01498629596755798</v>
       </c>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1157,6 +1187,8 @@
       <c r="R12" t="n">
         <v>0.005932908313592932</v>
       </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1215,6 +1247,8 @@
       <c r="R13" t="n">
         <v>0.02496931730419817</v>
       </c>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1273,6 +1307,8 @@
       <c r="R14" t="n">
         <v>0.04216014649383777</v>
       </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1327,6 +1363,8 @@
       <c r="R15" t="n">
         <v>0.04465261233339038</v>
       </c>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1381,6 +1419,8 @@
       <c r="R16" t="n">
         <v>0.046444056459004</v>
       </c>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1435,6 +1475,8 @@
       <c r="R17" t="n">
         <v>0.0426971189543995</v>
       </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1489,6 +1531,8 @@
       <c r="R18" t="n">
         <v>0.02547267761211013</v>
       </c>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1543,6 +1587,8 @@
       <c r="R19" t="n">
         <v>0.07412415624564839</v>
       </c>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1597,6 +1643,8 @@
       <c r="R20" t="n">
         <v>0.02982949637940507</v>
       </c>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1651,6 +1699,8 @@
       <c r="R21" t="n">
         <v>0.04775576276599745</v>
       </c>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1705,6 +1755,8 @@
       <c r="R22" t="n">
         <v>0.07178272167197755</v>
       </c>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1763,6 +1815,8 @@
       <c r="R23" t="n">
         <v>0.01940908164067787</v>
       </c>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1821,6 +1875,8 @@
       <c r="R24" t="n">
         <v>0.01112326027637736</v>
       </c>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1879,6 +1935,8 @@
       <c r="R25" t="n">
         <v>0.01940908164067787</v>
       </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1937,6 +1995,8 @@
       <c r="R26" t="n">
         <v>0.01940908164067787</v>
       </c>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1995,6 +2055,8 @@
       <c r="R27" t="n">
         <v>0.01112326027637736</v>
       </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2053,6 +2115,8 @@
       <c r="R28" t="n">
         <v>0.01112326027637736</v>
       </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2111,6 +2175,8 @@
       <c r="R29" t="n">
         <v>0.01718248205627023</v>
       </c>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2169,6 +2235,8 @@
       <c r="R30" t="n">
         <v>0.01718248205627023</v>
       </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2227,6 +2295,8 @@
       <c r="R31" t="n">
         <v>0.026548026103587</v>
       </c>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2285,6 +2355,8 @@
       <c r="R32" t="n">
         <v>0.01006019797878372</v>
       </c>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2343,6 +2415,8 @@
       <c r="R33" t="n">
         <v>0.02760079309767969</v>
       </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2401,6 +2475,8 @@
       <c r="R34" t="n">
         <v>0.02760079309767969</v>
       </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2459,6 +2535,8 @@
       <c r="R35" t="n">
         <v>0.03545959297481422</v>
       </c>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2517,6 +2595,8 @@
       <c r="R36" t="n">
         <v>0.03545959297481422</v>
       </c>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2575,6 +2655,8 @@
       <c r="R37" t="n">
         <v>0.03245576114304535</v>
       </c>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2633,6 +2715,8 @@
       <c r="R38" t="n">
         <v>0.04533517937991077</v>
       </c>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2691,6 +2775,8 @@
       <c r="R39" t="n">
         <v>0</v>
       </c>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2749,6 +2835,8 @@
       <c r="R40" t="n">
         <v>0.03679390372207091</v>
       </c>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2807,6 +2895,8 @@
       <c r="R41" t="n">
         <v>0.01940908164067787</v>
       </c>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2865,6 +2955,8 @@
       <c r="R42" t="n">
         <v>0.01112326027637736</v>
       </c>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2923,6 +3015,8 @@
       <c r="R43" t="n">
         <v>0.026548026103587</v>
       </c>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2981,6 +3075,8 @@
       <c r="R44" t="n">
         <v>0.02760079309767969</v>
       </c>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3039,6 +3135,8 @@
       <c r="R45" t="n">
         <v>0.03545959297481422</v>
       </c>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3097,6 +3195,8 @@
       <c r="R46" t="n">
         <v>0.05651580495753514</v>
       </c>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3155,6 +3255,8 @@
       <c r="R47" t="n">
         <v>0.06892894485763129</v>
       </c>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3213,6 +3315,8 @@
       <c r="R48" t="n">
         <v>0.0564584969409441</v>
       </c>
+      <c r="S48" t="inlineStr"/>
+      <c r="T48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3271,6 +3375,8 @@
       <c r="R49" t="n">
         <v>0.01365818713970217</v>
       </c>
+      <c r="S49" t="inlineStr"/>
+      <c r="T49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3329,6 +3435,8 @@
       <c r="R50" t="n">
         <v>0.04014487764849362</v>
       </c>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3387,6 +3495,8 @@
       <c r="R51" t="n">
         <v>0.01365818713970217</v>
       </c>
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3445,6 +3555,8 @@
       <c r="R52" t="n">
         <v>0.01365818713970217</v>
       </c>
+      <c r="S52" t="inlineStr"/>
+      <c r="T52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3503,6 +3615,8 @@
       <c r="R53" t="n">
         <v>0.01365818713970217</v>
       </c>
+      <c r="S53" t="inlineStr"/>
+      <c r="T53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3561,6 +3675,8 @@
       <c r="R54" t="n">
         <v>0.01365818713970217</v>
       </c>
+      <c r="S54" t="inlineStr"/>
+      <c r="T54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3619,6 +3735,8 @@
       <c r="R55" t="n">
         <v>0.04436113289559018</v>
       </c>
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3677,6 +3795,8 @@
       <c r="R56" t="n">
         <v>0.01123694784910104</v>
       </c>
+      <c r="S56" t="inlineStr"/>
+      <c r="T56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3735,6 +3855,8 @@
       <c r="R57" t="n">
         <v>0.005258692579715008</v>
       </c>
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3793,6 +3915,8 @@
       <c r="R58" t="n">
         <v>0.02614780329723496</v>
       </c>
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3851,6 +3975,8 @@
       <c r="R59" t="n">
         <v>0.02981974036652465</v>
       </c>
+      <c r="S59" t="inlineStr"/>
+      <c r="T59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3909,6 +4035,8 @@
       <c r="R60" t="n">
         <v>0.01882708618980631</v>
       </c>
+      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3967,6 +4095,8 @@
       <c r="R61" t="n">
         <v>0.005258692579715008</v>
       </c>
+      <c r="S61" t="inlineStr"/>
+      <c r="T61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4025,6 +4155,8 @@
       <c r="R62" t="n">
         <v>0.03172842995302576</v>
       </c>
+      <c r="S62" t="inlineStr"/>
+      <c r="T62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4083,6 +4215,8 @@
       <c r="R63" t="n">
         <v>0.02289970628700663</v>
       </c>
+      <c r="S63" t="inlineStr"/>
+      <c r="T63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4141,6 +4275,8 @@
       <c r="R64" t="n">
         <v>0.03762011370266357</v>
       </c>
+      <c r="S64" t="inlineStr"/>
+      <c r="T64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4199,6 +4335,8 @@
       <c r="R65" t="n">
         <v>0.01000636959259894</v>
       </c>
+      <c r="S65" t="inlineStr"/>
+      <c r="T65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4257,6 +4395,8 @@
       <c r="R66" t="n">
         <v>0.03922935157531927</v>
       </c>
+      <c r="S66" t="inlineStr"/>
+      <c r="T66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4315,6 +4455,8 @@
       <c r="R67" t="n">
         <v>0.03932005167897431</v>
       </c>
+      <c r="S67" t="inlineStr"/>
+      <c r="T67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4373,6 +4515,8 @@
       <c r="R68" t="n">
         <v>0.04958508262701199</v>
       </c>
+      <c r="S68" t="inlineStr"/>
+      <c r="T68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4431,6 +4575,8 @@
       <c r="R69" t="n">
         <v>0.05733476336399203</v>
       </c>
+      <c r="S69" t="inlineStr"/>
+      <c r="T69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4489,6 +4635,8 @@
       <c r="R70" t="n">
         <v>0.02880027709289949</v>
       </c>
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4547,6 +4695,8 @@
       <c r="R71" t="n">
         <v>0.04774613509449457</v>
       </c>
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4605,6 +4755,8 @@
       <c r="R72" t="n">
         <v>0.0286304818249801</v>
       </c>
+      <c r="S72" t="inlineStr"/>
+      <c r="T72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4663,6 +4815,8 @@
       <c r="R73" t="n">
         <v>0.01313746755009773</v>
       </c>
+      <c r="S73" t="inlineStr"/>
+      <c r="T73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4721,6 +4875,8 @@
       <c r="R74" t="n">
         <v>0.04353320095644261</v>
       </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4779,6 +4935,8 @@
       <c r="R75" t="n">
         <v>0.05036916693012583</v>
       </c>
+      <c r="S75" t="inlineStr"/>
+      <c r="T75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4837,6 +4995,8 @@
       <c r="R76" t="n">
         <v>0.09151655161265683</v>
       </c>
+      <c r="S76" t="inlineStr"/>
+      <c r="T76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4895,6 +5055,8 @@
       <c r="R77" t="n">
         <v>0.05069506281368039</v>
       </c>
+      <c r="S77" t="inlineStr"/>
+      <c r="T77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4953,6 +5115,8 @@
       <c r="R78" t="n">
         <v>0.0186604029259421</v>
       </c>
+      <c r="S78" t="inlineStr"/>
+      <c r="T78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5011,6 +5175,8 @@
       <c r="R79" t="n">
         <v>0.1275246570843699</v>
       </c>
+      <c r="S79" t="inlineStr"/>
+      <c r="T79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5069,6 +5235,8 @@
       <c r="R80" t="n">
         <v>0.1225743953061023</v>
       </c>
+      <c r="S80" t="inlineStr"/>
+      <c r="T80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5127,6 +5295,8 @@
       <c r="R81" t="n">
         <v>0.06567524429238983</v>
       </c>
+      <c r="S81" t="inlineStr"/>
+      <c r="T81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5185,6 +5355,8 @@
       <c r="R82" t="n">
         <v>0.05651580495753514</v>
       </c>
+      <c r="S82" t="inlineStr"/>
+      <c r="T82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5243,6 +5415,8 @@
       <c r="R83" t="n">
         <v>0</v>
       </c>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5301,6 +5475,8 @@
       <c r="R84" t="n">
         <v>0.09151655161265683</v>
       </c>
+      <c r="S84" t="inlineStr"/>
+      <c r="T84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5359,6 +5535,8 @@
       <c r="R85" t="n">
         <v>0.07357891121034246</v>
       </c>
+      <c r="S85" t="inlineStr"/>
+      <c r="T85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5417,6 +5595,8 @@
       <c r="R86" t="n">
         <v>0.07357891121034246</v>
       </c>
+      <c r="S86" t="inlineStr"/>
+      <c r="T86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5475,6 +5655,8 @@
       <c r="R87" t="n">
         <v>0.05069506281368039</v>
       </c>
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5533,6 +5715,8 @@
       <c r="R88" t="n">
         <v>0.02962769103852985</v>
       </c>
+      <c r="S88" t="inlineStr"/>
+      <c r="T88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5591,6 +5775,8 @@
       <c r="R89" t="n">
         <v>0.07056928534311084</v>
       </c>
+      <c r="S89" t="inlineStr"/>
+      <c r="T89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5649,6 +5835,8 @@
       <c r="R90" t="n">
         <v>0.02453009805722536</v>
       </c>
+      <c r="S90" t="inlineStr"/>
+      <c r="T90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5707,6 +5895,8 @@
       <c r="R91" t="n">
         <v>0.04323375905162748</v>
       </c>
+      <c r="S91" t="inlineStr"/>
+      <c r="T91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5765,6 +5955,8 @@
       <c r="R92" t="n">
         <v>0.06120548340203817</v>
       </c>
+      <c r="S92" t="inlineStr"/>
+      <c r="T92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5823,6 +6015,8 @@
       <c r="R93" t="n">
         <v>0.01810625476685216</v>
       </c>
+      <c r="S93" t="inlineStr"/>
+      <c r="T93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5881,6 +6075,8 @@
       <c r="R94" t="n">
         <v>0.01582119638561543</v>
       </c>
+      <c r="S94" t="inlineStr"/>
+      <c r="T94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5939,6 +6135,8 @@
       <c r="R95" t="n">
         <v>0.09499362880770693</v>
       </c>
+      <c r="S95" t="inlineStr"/>
+      <c r="T95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5997,6 +6195,8 @@
       <c r="R96" t="n">
         <v>0.1484065254011023</v>
       </c>
+      <c r="S96" t="inlineStr"/>
+      <c r="T96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6055,6 +6255,8 @@
       <c r="R97" t="n">
         <v>0.04338741584450634</v>
       </c>
+      <c r="S97" t="inlineStr"/>
+      <c r="T97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6113,6 +6315,8 @@
       <c r="R98" t="n">
         <v>0.03034497385943204</v>
       </c>
+      <c r="S98" t="inlineStr"/>
+      <c r="T98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6171,6 +6375,8 @@
       <c r="R99" t="n">
         <v>0.06010758751431648</v>
       </c>
+      <c r="S99" t="inlineStr"/>
+      <c r="T99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6229,6 +6435,8 @@
       <c r="R100" t="n">
         <v>0.01792827326992585</v>
       </c>
+      <c r="S100" t="inlineStr"/>
+      <c r="T100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6287,6 +6495,8 @@
       <c r="R101" t="n">
         <v>0.06010758751431648</v>
       </c>
+      <c r="S101" t="inlineStr"/>
+      <c r="T101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6345,6 +6555,8 @@
       <c r="R102" t="n">
         <v>0.01792827326992585</v>
       </c>
+      <c r="S102" t="inlineStr"/>
+      <c r="T102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6403,6 +6615,8 @@
       <c r="R103" t="n">
         <v>0.01175603153386143</v>
       </c>
+      <c r="S103" t="inlineStr"/>
+      <c r="T103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6461,6 +6675,8 @@
       <c r="R104" t="n">
         <v>0.04610789895390428</v>
       </c>
+      <c r="S104" t="inlineStr"/>
+      <c r="T104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6519,6 +6735,8 @@
       <c r="R105" t="n">
         <v>0.01228302606188206</v>
       </c>
+      <c r="S105" t="inlineStr"/>
+      <c r="T105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6577,6 +6795,8 @@
       <c r="R106" t="n">
         <v>0</v>
       </c>
+      <c r="S106" t="inlineStr"/>
+      <c r="T106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6635,6 +6855,8 @@
       <c r="R107" t="n">
         <v>0.03034497385943204</v>
       </c>
+      <c r="S107" t="inlineStr"/>
+      <c r="T107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6693,6 +6915,8 @@
       <c r="R108" t="n">
         <v>0.07138554373540211</v>
       </c>
+      <c r="S108" t="inlineStr"/>
+      <c r="T108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6751,6 +6975,8 @@
       <c r="R109" t="n">
         <v>0.04245189735119193</v>
       </c>
+      <c r="S109" t="inlineStr"/>
+      <c r="T109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6809,6 +7035,8 @@
       <c r="R110" t="n">
         <v>0.03019185147198399</v>
       </c>
+      <c r="S110" t="inlineStr"/>
+      <c r="T110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6867,6 +7095,8 @@
       <c r="R111" t="n">
         <v>0.04245189735119193</v>
       </c>
+      <c r="S111" t="inlineStr"/>
+      <c r="T111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6925,6 +7155,8 @@
       <c r="R112" t="n">
         <v>0.03019185147198399</v>
       </c>
+      <c r="S112" t="inlineStr"/>
+      <c r="T112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6983,6 +7215,8 @@
       <c r="R113" t="n">
         <v>0.03357979512793006</v>
       </c>
+      <c r="S113" t="inlineStr"/>
+      <c r="T113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7041,6 +7275,8 @@
       <c r="R114" t="n">
         <v>0.04367110333624002</v>
       </c>
+      <c r="S114" t="inlineStr"/>
+      <c r="T114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7099,6 +7335,8 @@
       <c r="R115" t="n">
         <v>0.005920755329285242</v>
       </c>
+      <c r="S115" t="inlineStr"/>
+      <c r="T115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7157,6 +7395,8 @@
       <c r="R116" t="n">
         <v>0.03583267613861628</v>
       </c>
+      <c r="S116" t="inlineStr"/>
+      <c r="T116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -7214,6 +7454,732 @@
       </c>
       <c r="R117" t="n">
         <v>0.03034497385943204</v>
+      </c>
+      <c r="S117" t="inlineStr"/>
+      <c r="T117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C118" t="n">
+        <v>22</v>
+      </c>
+      <c r="D118" t="n">
+        <v>3</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0.7944444616635641</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0.745261569817861</v>
+      </c>
+      <c r="G118" t="n">
+        <v>0.1027658134698868</v>
+      </c>
+      <c r="H118" t="n">
+        <v>0.7222222487131754</v>
+      </c>
+      <c r="I118" t="n">
+        <v>0.5860305825869242</v>
+      </c>
+      <c r="J118" t="n">
+        <v>0.0207181076124321</v>
+      </c>
+      <c r="K118" t="n">
+        <v>0.01746491577653433</v>
+      </c>
+      <c r="L118" t="n">
+        <v>0.00506271653945393</v>
+      </c>
+      <c r="M118" t="n">
+        <v>0.007856734520410793</v>
+      </c>
+      <c r="N118" t="n">
+        <v>0.005126155402093149</v>
+      </c>
+      <c r="O118" t="n">
+        <v>0.7222222487131754</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0.007856734520410793</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0.7408978541692098</v>
+      </c>
+      <c r="R118" t="n">
+        <v>0.03034497385943204</v>
+      </c>
+      <c r="S118" t="inlineStr"/>
+      <c r="T118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Image_binary</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C119" t="n">
+        <v>22</v>
+      </c>
+      <c r="D119" t="n">
+        <v>3</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0.5444444616635641</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.4536264847106394</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I119" t="n">
+        <v>0.3696845471858978</v>
+      </c>
+      <c r="J119" t="n">
+        <v>0.1429522376603718</v>
+      </c>
+      <c r="K119" t="n">
+        <v>0.1275516061403077</v>
+      </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
+      <c r="M119" t="n">
+        <v>0.09736101612758238</v>
+      </c>
+      <c r="N119" t="n">
+        <v>0.07879416312299103</v>
+      </c>
+      <c r="O119" t="n">
+        <v>0.6166666646798452</v>
+      </c>
+      <c r="P119" t="n">
+        <v>0.2494438215369265</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>0.2764622817436854</v>
+      </c>
+      <c r="R119" t="n">
+        <v>0.0447275802481077</v>
+      </c>
+      <c r="S119" t="inlineStr"/>
+      <c r="T119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Image_binary</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C120" t="n">
+        <v>22</v>
+      </c>
+      <c r="D120" t="n">
+        <v>3</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0.6030555566151937</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0.4111700783421784</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="n">
+        <v>0.6583333214124044</v>
+      </c>
+      <c r="I120" t="n">
+        <v>0.3275231768687566</v>
+      </c>
+      <c r="J120" t="n">
+        <v>0.04247183566551653</v>
+      </c>
+      <c r="K120" t="n">
+        <v>0.02492560627937922</v>
+      </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
+      <c r="M120" t="n">
+        <v>0.1234627534221223</v>
+      </c>
+      <c r="N120" t="n">
+        <v>0.1088146377908272</v>
+      </c>
+      <c r="O120" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="P120" t="n">
+        <v>0.1312334592680055</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>0.378510390718778</v>
+      </c>
+      <c r="R120" t="n">
+        <v>0.1426953046710271</v>
+      </c>
+      <c r="S120" t="inlineStr"/>
+      <c r="T120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Image_binary</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C121" t="n">
+        <v>22</v>
+      </c>
+      <c r="D121" t="n">
+        <v>3</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0.6030555566151937</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.4111700783421784</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="n">
+        <v>0.6583333214124044</v>
+      </c>
+      <c r="I121" t="n">
+        <v>0.3275231768687566</v>
+      </c>
+      <c r="J121" t="n">
+        <v>0.04247183566551653</v>
+      </c>
+      <c r="K121" t="n">
+        <v>0.02492560627937922</v>
+      </c>
+      <c r="L121" t="n">
+        <v>0</v>
+      </c>
+      <c r="M121" t="n">
+        <v>0.1234627534221223</v>
+      </c>
+      <c r="N121" t="n">
+        <v>0.1088146377908272</v>
+      </c>
+      <c r="O121" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="P121" t="n">
+        <v>0.1312334592680055</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>0.378510390718778</v>
+      </c>
+      <c r="R121" t="n">
+        <v>0.1426953046710271</v>
+      </c>
+      <c r="S121" t="inlineStr"/>
+      <c r="T121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Image_binary</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C122" t="n">
+        <v>22</v>
+      </c>
+      <c r="D122" t="n">
+        <v>3</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.6030555566151937</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0.4111700783421784</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0.6583333214124044</v>
+      </c>
+      <c r="I122" t="n">
+        <v>0.3275231768687566</v>
+      </c>
+      <c r="J122" t="n">
+        <v>0.04247183566551653</v>
+      </c>
+      <c r="K122" t="n">
+        <v>0.02492560627937922</v>
+      </c>
+      <c r="L122" t="n">
+        <v>0</v>
+      </c>
+      <c r="M122" t="n">
+        <v>0.1234627534221223</v>
+      </c>
+      <c r="N122" t="n">
+        <v>0.1088146377908272</v>
+      </c>
+      <c r="O122" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="P122" t="n">
+        <v>0.1312334592680055</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>0.378510390718778</v>
+      </c>
+      <c r="R122" t="n">
+        <v>0.1426953046710271</v>
+      </c>
+      <c r="S122" t="inlineStr"/>
+      <c r="T122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Image_binary</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C123" t="n">
+        <v>22</v>
+      </c>
+      <c r="D123" t="n">
+        <v>3</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0.6030555566151937</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0.4111700783421784</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="n">
+        <v>0.6583333214124044</v>
+      </c>
+      <c r="I123" t="n">
+        <v>0.3275231768687566</v>
+      </c>
+      <c r="J123" t="n">
+        <v>0.04247183566551653</v>
+      </c>
+      <c r="K123" t="n">
+        <v>0.02492560627937922</v>
+      </c>
+      <c r="L123" t="n">
+        <v>0</v>
+      </c>
+      <c r="M123" t="n">
+        <v>0.1234627534221223</v>
+      </c>
+      <c r="N123" t="n">
+        <v>0.1088146377908272</v>
+      </c>
+      <c r="O123" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="P123" t="n">
+        <v>0.1312334592680055</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>0.378510390718778</v>
+      </c>
+      <c r="R123" t="n">
+        <v>0.1426953046710271</v>
+      </c>
+      <c r="S123" t="inlineStr"/>
+      <c r="T123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C124" t="n">
+        <v>22</v>
+      </c>
+      <c r="D124" t="n">
+        <v>3</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.7033106088638306</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
+      <c r="I124" t="n">
+        <v>0</v>
+      </c>
+      <c r="J124" t="n">
+        <v>0</v>
+      </c>
+      <c r="K124" t="n">
+        <v>0.01581045943116539</v>
+      </c>
+      <c r="L124" t="n">
+        <v>0</v>
+      </c>
+      <c r="M124" t="n">
+        <v>0</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+      <c r="P124" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>0</v>
+      </c>
+      <c r="R124" t="n">
+        <v>0</v>
+      </c>
+      <c r="S124" t="inlineStr"/>
+      <c r="T124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C125" t="n">
+        <v>22</v>
+      </c>
+      <c r="D125" t="n">
+        <v>3</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.7033106088638306</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
+      <c r="I125" t="n">
+        <v>0</v>
+      </c>
+      <c r="J125" t="n">
+        <v>0</v>
+      </c>
+      <c r="K125" t="n">
+        <v>0.01581045943116539</v>
+      </c>
+      <c r="L125" t="n">
+        <v>0</v>
+      </c>
+      <c r="M125" t="n">
+        <v>0</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
+      <c r="P125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>0</v>
+      </c>
+      <c r="R125" t="n">
+        <v>0</v>
+      </c>
+      <c r="S125" t="inlineStr"/>
+      <c r="T125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C126" t="n">
+        <v>22</v>
+      </c>
+      <c r="D126" t="n">
+        <v>3</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.6166287561257681</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0.1433352927366892</v>
+      </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
+      <c r="I126" t="n">
+        <v>0</v>
+      </c>
+      <c r="J126" t="n">
+        <v>0</v>
+      </c>
+      <c r="K126" t="n">
+        <v>0.1754909601564643</v>
+      </c>
+      <c r="L126" t="n">
+        <v>0.006886877055669918</v>
+      </c>
+      <c r="M126" t="n">
+        <v>0</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+      <c r="P126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" t="n">
+        <v>0</v>
+      </c>
+      <c r="S126" t="inlineStr"/>
+      <c r="T126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C127" t="n">
+        <v>22</v>
+      </c>
+      <c r="D127" t="n">
+        <v>3</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0.7033106088638306</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0.1027658134698868</v>
+      </c>
+      <c r="H127" t="n">
+        <v>0</v>
+      </c>
+      <c r="I127" t="n">
+        <v>0</v>
+      </c>
+      <c r="J127" t="n">
+        <v>0</v>
+      </c>
+      <c r="K127" t="n">
+        <v>0.01581045943116539</v>
+      </c>
+      <c r="L127" t="n">
+        <v>0.00506271653945393</v>
+      </c>
+      <c r="M127" t="n">
+        <v>0</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
+      <c r="P127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>0</v>
+      </c>
+      <c r="R127" t="n">
+        <v>0</v>
+      </c>
+      <c r="S127" t="inlineStr"/>
+      <c r="T127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C128" t="n">
+        <v>22</v>
+      </c>
+      <c r="D128" t="n">
+        <v>3</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0.7033106088638306</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0.1027658134698868</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="n">
+        <v>0</v>
+      </c>
+      <c r="J128" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" t="n">
+        <v>0.01581045943116539</v>
+      </c>
+      <c r="L128" t="n">
+        <v>0.00506271653945393</v>
+      </c>
+      <c r="M128" t="n">
+        <v>0</v>
+      </c>
+      <c r="N128" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0</v>
+      </c>
+      <c r="P128" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>0</v>
+      </c>
+      <c r="R128" t="n">
+        <v>0</v>
+      </c>
+      <c r="S128" t="inlineStr"/>
+      <c r="T128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Image_only</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="C129" t="n">
+        <v>22</v>
+      </c>
+      <c r="D129" t="n">
+        <v>3</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0.7033106088638306</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0.1027658134698868</v>
+      </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="n">
+        <v>0</v>
+      </c>
+      <c r="J129" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" t="n">
+        <v>0.01581045943116539</v>
+      </c>
+      <c r="L129" t="n">
+        <v>0.00506271653945393</v>
+      </c>
+      <c r="M129" t="n">
+        <v>0</v>
+      </c>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="n">
+        <v>0</v>
+      </c>
+      <c r="P129" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>0</v>
+      </c>
+      <c r="R129" t="n">
+        <v>0</v>
+      </c>
+      <c r="S129" t="n">
+        <v>0.6871217290560404</v>
+      </c>
+      <c r="T129" t="n">
+        <v>0.02029802562326791</v>
       </c>
     </row>
   </sheetData>

</xml_diff>